<commit_message>
fixed number error in sprint backlog
</commit_message>
<xml_diff>
--- a/presentations/links/sprintbacklog1.xlsx
+++ b/presentations/links/sprintbacklog1.xlsx
@@ -275,20 +275,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="27">
@@ -375,7 +375,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -484,7 +483,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -643,7 +641,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -740,11 +737,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="-727094272"/>
-        <c:axId val="-710638576"/>
+        <c:axId val="-705604208"/>
+        <c:axId val="-705272176"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-727094272"/>
+        <c:axId val="-705604208"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -776,7 +773,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -843,7 +839,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-710638576"/>
+        <c:crossAx val="-705272176"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -851,7 +847,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-710638576"/>
+        <c:axId val="-705272176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -909,7 +905,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -970,7 +965,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-727094272"/>
+        <c:crossAx val="-705604208"/>
         <c:crossesAt val="1.0"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -984,7 +979,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:solidFill>
@@ -2064,7 +2058,7 @@
       <c r="Q1" s="2"/>
     </row>
     <row r="2" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="13">
+      <c r="A2" s="10">
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
@@ -2087,7 +2081,7 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A3" s="13"/>
+      <c r="A3" s="10"/>
       <c r="B3" s="12"/>
       <c r="C3" s="4">
         <v>2</v>
@@ -2109,7 +2103,7 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A4" s="13"/>
+      <c r="A4" s="10"/>
       <c r="B4" s="12"/>
       <c r="C4" s="4">
         <v>3</v>
@@ -2131,7 +2125,7 @@
       </c>
     </row>
     <row r="5" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="13"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="12"/>
       <c r="C5" s="4">
         <v>4</v>
@@ -2150,7 +2144,7 @@
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.15">
-      <c r="A6" s="13"/>
+      <c r="A6" s="10"/>
       <c r="B6" s="12"/>
       <c r="C6" s="4">
         <v>5</v>
@@ -2169,7 +2163,7 @@
       </c>
     </row>
     <row r="7" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A7" s="13"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="12"/>
       <c r="C7" s="4">
         <v>6</v>
@@ -2191,7 +2185,7 @@
       </c>
     </row>
     <row r="8" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A8" s="13"/>
+      <c r="A8" s="10"/>
       <c r="B8" s="12"/>
       <c r="C8" s="4">
         <v>7</v>
@@ -2216,7 +2210,7 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A9" s="13"/>
+      <c r="A9" s="10"/>
       <c r="B9" s="12"/>
       <c r="C9" s="4">
         <v>8</v>
@@ -2235,7 +2229,7 @@
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.15">
-      <c r="A10" s="13"/>
+      <c r="A10" s="10"/>
       <c r="B10" s="12"/>
       <c r="C10" s="4">
         <v>9</v>
@@ -2254,7 +2248,7 @@
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.15">
-      <c r="A11" s="13"/>
+      <c r="A11" s="10"/>
       <c r="B11" s="12"/>
       <c r="C11" s="5">
         <v>10</v>
@@ -2276,7 +2270,7 @@
       </c>
     </row>
     <row r="12" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A12" s="13"/>
+      <c r="A12" s="10"/>
       <c r="B12" s="12"/>
       <c r="C12" s="4">
         <v>11</v>
@@ -2289,14 +2283,14 @@
       </c>
     </row>
     <row r="13" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A13" s="13">
+      <c r="A13" s="10">
         <v>2</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="11" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="5">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>28</v>
@@ -2312,10 +2306,10 @@
       </c>
     </row>
     <row r="14" spans="1:17" ht="26" x14ac:dyDescent="0.15">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="11"/>
       <c r="C14" s="5">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>29</v>
@@ -2390,17 +2384,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2490,15 +2484,15 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
finished sprint 1, starting sprint2
</commit_message>
<xml_diff>
--- a/presentations/links/sprintbacklog1.xlsx
+++ b/presentations/links/sprintbacklog1.xlsx
@@ -9,13 +9,14 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="220" yWindow="460" windowWidth="28580" windowHeight="16740"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16740"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint1" sheetId="5" r:id="rId1"/>
     <sheet name="Burndown Chart" sheetId="6" r:id="rId2"/>
   </sheets>
   <calcPr calcId="150001" concurrentCalc="0"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="52">
   <si>
     <t>Task</t>
   </si>
@@ -160,6 +161,30 @@
   </si>
   <si>
     <t>Actual:</t>
+  </si>
+  <si>
+    <t>Detailed Description</t>
+  </si>
+  <si>
+    <t>using forms on html, using javascript for the submit button</t>
+  </si>
+  <si>
+    <t>use php to pass the data to the next html file that lists all created assignments</t>
+  </si>
+  <si>
+    <t>pictures for background, using forms, buttons, links on html</t>
+  </si>
+  <si>
+    <t>using mysql create database, create tables, setup user accounts</t>
+  </si>
+  <si>
+    <t>create sql query to insert into table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">create nav bar side bar, create css document for global side bar, </t>
+  </si>
+  <si>
+    <t>used html forms to input information, and input excel file using html forms, custom css for formatting</t>
   </si>
 </sst>
 </file>
@@ -278,26 +303,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="27">
@@ -384,6 +409,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -492,6 +518,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -650,6 +677,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -719,16 +747,16 @@
                   <c:v>12.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12.0</c:v>
+                  <c:v>7.0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12.0</c:v>
+                  <c:v>5.0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12.0</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12.0</c:v>
+                  <c:v>0.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -746,11 +774,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="-1017367232"/>
-        <c:axId val="-1017363472"/>
+        <c:axId val="856708960"/>
+        <c:axId val="856881056"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-1017367232"/>
+        <c:axId val="856708960"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -782,6 +810,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -848,7 +877,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1017363472"/>
+        <c:crossAx val="856881056"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -856,7 +885,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-1017363472"/>
+        <c:axId val="856881056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -914,6 +943,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -974,7 +1004,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1017367232"/>
+        <c:crossAx val="856708960"/>
         <c:crossesAt val="1.0"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -988,6 +1018,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:solidFill>
@@ -2003,29 +2034,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y17"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="53" style="4" customWidth="1"/>
     <col min="3" max="3" width="8" style="4" customWidth="1"/>
-    <col min="4" max="4" width="42.83203125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="2.83203125" style="8" customWidth="1"/>
-    <col min="8" max="8" width="13.5" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.33203125" style="11" customWidth="1"/>
-    <col min="10" max="10" width="5.83203125" style="1" customWidth="1"/>
-    <col min="11" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="6" style="1" customWidth="1"/>
-    <col min="16" max="16" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="3.6640625" style="8" customWidth="1"/>
-    <col min="18" max="18" width="7" style="12" customWidth="1"/>
-    <col min="19" max="25" width="6" style="1" customWidth="1"/>
-    <col min="26" max="16384" width="12" style="1"/>
+    <col min="4" max="5" width="42.83203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="2.83203125" style="8" customWidth="1"/>
+    <col min="9" max="9" width="13.5" style="1" customWidth="1"/>
+    <col min="10" max="10" width="11.33203125" style="10" customWidth="1"/>
+    <col min="11" max="11" width="5.83203125" style="1" customWidth="1"/>
+    <col min="12" max="13" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="6" style="1" customWidth="1"/>
+    <col min="17" max="17" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.6640625" style="8" customWidth="1"/>
+    <col min="19" max="19" width="7" style="9" customWidth="1"/>
+    <col min="20" max="26" width="6" style="1" customWidth="1"/>
+    <col min="27" max="16384" width="12" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:26" ht="75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2039,65 +2070,68 @@
         <v>0</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="S1" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="14">
+    <row r="2" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="11">
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
@@ -2109,18 +2143,24 @@
       <c r="D2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="1">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="E2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="O2" s="1">
+      <c r="P2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="26" x14ac:dyDescent="0.15">
-      <c r="A3" s="14"/>
+    <row r="3" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A3" s="11"/>
       <c r="B3" s="13"/>
       <c r="C3" s="4">
         <v>2</v>
@@ -2129,20 +2169,26 @@
         <v>31</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="1">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1" t="s">
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="P3" s="1">
-        <v>1</v>
+      <c r="Q3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="26" x14ac:dyDescent="0.15">
-      <c r="A4" s="14"/>
+    <row r="4" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A4" s="11"/>
       <c r="B4" s="13"/>
       <c r="C4" s="4">
         <v>3</v>
@@ -2151,20 +2197,26 @@
         <v>32</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="1">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1" t="s">
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="P4" s="1">
-        <v>1</v>
+      <c r="Q4" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="14"/>
+    <row r="5" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="11"/>
       <c r="B5" s="13"/>
       <c r="C5" s="4">
         <v>4</v>
@@ -2172,18 +2224,24 @@
       <c r="D5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="1">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1" t="s">
+      <c r="E5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M5" s="1">
+      <c r="N5" s="1">
+        <v>1</v>
+      </c>
+      <c r="W5" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.15">
-      <c r="A6" s="14"/>
+    <row r="6" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A6" s="11"/>
       <c r="B6" s="13"/>
       <c r="C6" s="4">
         <v>5</v>
@@ -2191,18 +2249,24 @@
       <c r="D6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="s">
+      <c r="E6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M6" s="1">
+      <c r="N6" s="1">
+        <v>1</v>
+      </c>
+      <c r="W6" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="26" x14ac:dyDescent="0.15">
-      <c r="A7" s="14"/>
+    <row r="7" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A7" s="11"/>
       <c r="B7" s="13"/>
       <c r="C7" s="4">
         <v>6</v>
@@ -2211,20 +2275,26 @@
         <v>21</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="1">
+      <c r="G7" s="1">
         <v>0.5</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M7" s="1">
+      <c r="N7" s="1">
         <v>0.5</v>
       </c>
+      <c r="W7" s="1">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="8" spans="1:25" ht="39" x14ac:dyDescent="0.15">
-      <c r="A8" s="14"/>
+    <row r="8" spans="1:26" ht="39" x14ac:dyDescent="0.15">
+      <c r="A8" s="11"/>
       <c r="B8" s="13"/>
       <c r="C8" s="4">
         <v>7</v>
@@ -2233,23 +2303,35 @@
         <v>41</v>
       </c>
       <c r="E8" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="1">
+      <c r="G8" s="1">
         <v>2</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N8" s="1">
-        <v>1</v>
-      </c>
       <c r="O8" s="1">
         <v>1</v>
       </c>
+      <c r="P8" s="1">
+        <v>1</v>
+      </c>
+      <c r="X8" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="1:25" ht="26" x14ac:dyDescent="0.15">
-      <c r="A9" s="14"/>
+    <row r="9" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A9" s="11"/>
       <c r="B9" s="13"/>
       <c r="C9" s="4">
         <v>8</v>
@@ -2257,18 +2339,24 @@
       <c r="D9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="1">
-        <v>1</v>
-      </c>
-      <c r="H9" s="1" t="s">
+      <c r="E9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
+      <c r="I9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M9" s="1">
+      <c r="N9" s="1">
+        <v>1</v>
+      </c>
+      <c r="W9" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.15">
-      <c r="A10" s="14"/>
+    <row r="10" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A10" s="11"/>
       <c r="B10" s="13"/>
       <c r="C10" s="4">
         <v>9</v>
@@ -2276,18 +2364,24 @@
       <c r="D10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="1">
-        <v>1</v>
-      </c>
-      <c r="H10" s="1" t="s">
+      <c r="E10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M10" s="1">
+      <c r="N10" s="1">
+        <v>1</v>
+      </c>
+      <c r="W10" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.15">
-      <c r="A11" s="14"/>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.15">
+      <c r="A11" s="11"/>
       <c r="B11" s="13"/>
       <c r="C11" s="5">
         <v>10</v>
@@ -2296,20 +2390,26 @@
         <v>22</v>
       </c>
       <c r="E11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="1">
+      <c r="G11" s="1">
         <v>0.5</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M11" s="1">
+      <c r="N11" s="1">
         <v>0.5</v>
       </c>
+      <c r="W11" s="1">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="12" spans="1:25" ht="26" x14ac:dyDescent="0.15">
-      <c r="A12" s="14"/>
+    <row r="12" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A12" s="11"/>
       <c r="B12" s="13"/>
       <c r="C12" s="4">
         <v>11</v>
@@ -2317,15 +2417,15 @@
       <c r="D12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="1">
+      <c r="G12" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="26" x14ac:dyDescent="0.15">
-      <c r="A13" s="14">
+    <row r="13" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A13" s="11">
         <v>2</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="12" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="5">
@@ -2334,78 +2434,86 @@
       <c r="D13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="1">
-        <v>1</v>
-      </c>
-      <c r="H13" s="1" t="s">
+      <c r="E13" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" s="1">
+        <v>1</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="N13" s="1">
+      <c r="O13" s="1">
+        <v>1</v>
+      </c>
+      <c r="X13" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="26" x14ac:dyDescent="0.15">
-      <c r="A14" s="14"/>
-      <c r="B14" s="15"/>
+    <row r="14" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+      <c r="A14" s="11"/>
+      <c r="B14" s="12"/>
       <c r="C14" s="5">
         <v>13</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="1">
-        <v>1</v>
-      </c>
-      <c r="H14" s="1" t="s">
+      <c r="E14" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="N14" s="1">
+      <c r="O14" s="1">
+        <v>1</v>
+      </c>
+      <c r="X14" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="6:25" x14ac:dyDescent="0.15">
-      <c r="F17" s="2">
-        <f>SUM(F2:F16)</f>
+    <row r="17" spans="7:26" x14ac:dyDescent="0.15">
+      <c r="G17" s="2">
+        <f>SUM(G2:G16)</f>
         <v>12</v>
       </c>
-      <c r="J17" s="2">
-        <f>SUM(J2:J14)</f>
+      <c r="K17" s="2">
+        <f>SUM(K2:K14)</f>
         <v>0</v>
       </c>
-      <c r="K17" s="2">
-        <f t="shared" ref="K17:P17" si="0">SUM(K2:K14)</f>
+      <c r="L17" s="2">
+        <f t="shared" ref="L17:Q17" si="0">SUM(L2:L14)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="2">
+      <c r="M17" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M17" s="2">
+      <c r="N17" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N17" s="2">
+      <c r="O17" s="2">
         <f t="shared" si="0"/>
         <v>3</v>
-      </c>
-      <c r="O17" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
       </c>
       <c r="P17" s="2">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="S17" s="2">
-        <f>SUM(S2:S14)</f>
+      <c r="Q17" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="T17" s="2">
+        <f>SUM(T2:T14)</f>
         <v>0</v>
       </c>
-      <c r="T17" s="2">
-        <f t="shared" ref="T17:Y17" si="1">SUM(T2:T14)</f>
-        <v>0</v>
-      </c>
       <c r="U17" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="U17:Z17" si="1">SUM(U2:U14)</f>
         <v>0</v>
       </c>
       <c r="V17" s="2">
@@ -2414,23 +2522,27 @@
       </c>
       <c r="W17" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X17" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y17" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="Z17" s="2">
+        <f t="shared" si="1"/>
+        <v>9.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="Q1:Q1048576"/>
     <mergeCell ref="R1:R1048576"/>
-    <mergeCell ref="I1:I1048576"/>
-    <mergeCell ref="G1:G1048576"/>
+    <mergeCell ref="S1:S1048576"/>
+    <mergeCell ref="J1:J1048576"/>
+    <mergeCell ref="H1:H1048576"/>
     <mergeCell ref="A13:A14"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="B2:B12"/>
@@ -2453,17 +2565,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2540,28 +2652,28 @@
         <v>12</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H4">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2574,7 +2686,65 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
 <xsd:schema targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f7c28edf12e174e47f2c7bd2736e8bd" ns2:_="" ns3:_="" ns4:_="" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d93dc7d-5998-434b-bf34-aa89b432ec07" xmlns:ns3="$ListId:Shared Documents;" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v4">
 <xsd:import namespace="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
 <xsd:import namespace="$ListId:Shared Documents;"/>
@@ -2748,65 +2918,35 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
+    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B9EEEF-7393-4E57-9716-D967A23AC816}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F807D2B-FCE5-4B63-BC9A-551BEF173D66}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0008E140-BD0E-4C41-947D-F18B1A1E4B6B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2824,32 +2964,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
-    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B9EEEF-7393-4E57-9716-D967A23AC816}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F807D2B-FCE5-4B63-BC9A-551BEF173D66}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>